<commit_message>
add: send image to telegram
</commit_message>
<xml_diff>
--- a/vehicle_data.xlsx
+++ b/vehicle_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1330,6 +1330,26 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>6</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2025-11-30 16:14:55</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: duplicate send message to tele
</commit_message>
<xml_diff>
--- a/vehicle_data.xlsx
+++ b/vehicle_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1350,6 +1350,1446 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>5</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>5</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>5</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>5</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>5</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>5</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>5</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>5</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>5</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>5</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>5</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>5</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>5</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>5</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>5</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>5</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>5</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>5</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>5</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>5</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>5</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>5</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>5</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>5</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>5</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>5</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>5</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>77A-247.01</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>2025-12-03 00:14:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>1</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:13:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>1</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>1</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>1</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>1</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>1</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>1</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>1</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>1</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>1</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>1</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>1</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>1</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>1</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>2025-12-03 11:16:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>1</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:46:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>1</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:46:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>1</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:46:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>1</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:46:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>1</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:46:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>1</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:46:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>1</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:46:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>1</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:46:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>1</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:46:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>1</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:46:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>1</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:49:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>1</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:49:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>1</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:49:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>1</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:49:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>1</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:49:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>1</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:49:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>1</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:49:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>1</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:52:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>1</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:52:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>1</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:52:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>1</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:52:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>1</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>2025-12-03 14:52:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>1</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>2025-12-03 15:53:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>1</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>2025-12-03 15:53:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>1</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>2025-12-03 15:53:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>1</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>2025-12-03 15:53:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>1</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>2025-12-03 15:53:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>1</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>2025-12-03 15:53:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>1</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>2025-12-03 15:53:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>1</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>77L-1003</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>2025-12-03 15:53:56</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>